<commit_message>
docs(#207): KBD-VI-ORDERFREE test cases + spec results appendix
VIOF-1..19 cover the Samsung study rows, every mark ordering, the three
divergence classes the matrix found, and the two must-not-regress gates.
The spec appendix records the 43,791-case result, the fixes, and the two
deliberate non-parity calls (unreachable uơ, modern tone placement).
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -29,6 +29,7 @@
     <sheet name="KBD-CJK-CYCLE" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="KBD-ZH-PINYIN" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="KBD-JP-FLICK" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="KBD-VI-ORDERFREE" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5996,6 +5997,16 @@
   </sheetPr>
   <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8292,6 +8303,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VIOF-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tone typed before horn</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>type t,u,o,n,g,r,w</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>field shows "tưởng" (Samsung parity)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests; device 2026-09-11</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VIOF-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Horn typed before tone (existing order)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>type t,u,o,n,g,w,r</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>"tưởng" — must not regress</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VIOF-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tone before horn on a 3-vowel nucleus</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>type n,g,u,o,i,f,w</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>"người"</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests; device 2026-09-11</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>VIOF-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tone moves onto the newly horned vowel</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>type m,u,a,s,w</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>"mứa" — tone follows the ư, not left on u</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VIOF-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tone typed before a late circumflex</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>type c,a,n,s,j,a</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>"cận"</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VIOF-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Circumflex after tone, behind a coda</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>type d,d,o,n,g,f,o</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>"đồng"</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VIOF-7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Horn replaces an existing circumflex</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>type o,o,w</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>"ơ" — w overrides ô</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VIOF-8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Circumflex replaces an existing horn</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>type o,w,o</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>"ô" — o overrides ơ</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VIOF-9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Remote đ: trailing d marks the d-initial</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>type d,u,o,c,d</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>"đuoc" — initial becomes đ</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>VIOF-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Remote đ + horn + tone, any order</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>type duoc then any permutation of d,w,j</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>"được" for all 6 orderings</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests; device 2026-09-11</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>VIOF-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Remote đ preserves the initial's case</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>VI pack, shift on first key</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>type D,u,o,c,d,w,j</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>"Được"</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>VIOF-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Remote đ after a tone</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>type d,u,n,g,f,d</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>"đùng"</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VIOF-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Second remote d reverts</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>type d,u,o,c,d,d</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>"duocd" — đ reverted, d literal</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>VIOF-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Trailing d stays literal without a d initial</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>type b,a,d</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>"bad" untouched</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>VIOF-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Horn reaches the nucleus over an offglide</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>type g,u,i,w / type c,u,u,w</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>"gưi" / "cưu" — not "guiw"/"cuư"</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>VIOF-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Circumflex after tone auto-promotion is idempotent</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>type i,e,c,s,e</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>"iếc" — the e does not cancel the promoted ê</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>VIOF-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>qu/gi glide never takes the horn</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>type q,u,o,w,f</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>"quờ" — not "qừo"</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>TelexOrderVectorsTest/Tests + TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>VIOF-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Every valid syllable in every mark order</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>run the generated matrix (43k cases) on both ports</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>zero divergences</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>TelexExhaustiveTest/Tests</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>VIOF-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Existing Telex behaviour unchanged</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>run the full Telex suite both platforms</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>324 Kotlin + 291 Swift tests green</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>CI mobile-test-ci + mobile-swift-ci</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>